<commit_message>
added order data merging script
</commit_message>
<xml_diff>
--- a/data/simulation_high_frequency_tier.xlsx
+++ b/data/simulation_high_frequency_tier.xlsx
@@ -8,26 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wei.kc\Desktop\Adhoc\03 Sept 2026\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2C2F6D7-DF4A-42A6-8CD5-9CC0FD82D7A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7BEF59E-86ED-49BD-A8EE-3B7737AD03AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="826" activeTab="7" xr2:uid="{2FEC0780-5ED5-45AE-9712-E8F411AADB37}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="826" activeTab="6" xr2:uid="{2FEC0780-5ED5-45AE-9712-E8F411AADB37}"/>
   </bookViews>
   <sheets>
     <sheet name="July 2026 " sheetId="1" r:id="rId1"/>
     <sheet name="&gt;50% order(July)" sheetId="3" r:id="rId2"/>
     <sheet name="Aug 2026" sheetId="2" r:id="rId3"/>
     <sheet name="&gt;50% order(Aug)" sheetId="4" r:id="rId4"/>
-    <sheet name="16 Accounts given" sheetId="5" r:id="rId5"/>
-    <sheet name="account to check (July)" sheetId="6" r:id="rId6"/>
-    <sheet name="account to check(Aug)" sheetId="7" r:id="rId7"/>
-    <sheet name="unique id" sheetId="8" r:id="rId8"/>
+    <sheet name="Sheet1" sheetId="9" r:id="rId5"/>
+    <sheet name="16 Accounts given" sheetId="5" r:id="rId6"/>
+    <sheet name="account to check (July)" sheetId="6" r:id="rId7"/>
+    <sheet name="account to check(Aug)" sheetId="7" r:id="rId8"/>
+    <sheet name="unique id" sheetId="8" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'&gt;50% order(Aug)'!$A$1:$J$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'&gt;50% order(July)'!$A$1:$J$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Aug 2026'!$A$1:$I$455</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'July 2026 '!$A$1:$I$375</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'unique id'!$A$1:$C$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'unique id'!$A$1:$C$43</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="86">
   <si>
     <t>user_id</t>
   </si>
@@ -237,6 +238,82 @@
   <si>
     <t>year</t>
   </si>
+  <si>
+    <t>July &amp;  Aug 2026</t>
+  </si>
+  <si>
+    <t>Order creation lag</t>
+  </si>
+  <si>
+    <t>Parameter</t>
+  </si>
+  <si>
+    <t>High frequency volume share</t>
+  </si>
+  <si>
+    <t>&gt; 50% of total orders</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Evaluation Window</t>
+  </si>
+  <si>
+    <t>Enforcement Trigger</t>
+  </si>
+  <si>
+    <t>Action Taken</t>
+  </si>
+  <si>
+    <t>Suggestion:</t>
+  </si>
+  <si>
+    <t>Analysis period</t>
+  </si>
+  <si>
+    <t>&lt; 30 seconds</t>
+  </si>
+  <si>
+    <t>1-hour rolling window (3600 seconds)</t>
+  </si>
+  <si>
+    <t>Order placing block</t>
+  </si>
+  <si>
+    <t>Strategy  conditions</t>
+  </si>
+  <si>
+    <t>Rule Threshold/Value</t>
+  </si>
+  <si>
+    <t>&gt;5 high-frequency orders</t>
+  </si>
+  <si>
+    <t>Flagging criteria</t>
+  </si>
+  <si>
+    <t>More than 3 flag in 1-hour rolling window
+HF share &gt;50% of total orders</t>
+  </si>
+  <si>
+    <t>Evaluation dimension</t>
+  </si>
+  <si>
+    <t>Flagged</t>
+  </si>
+  <si>
+    <t>Direct accounts</t>
+  </si>
+  <si>
+    <t>Already banned</t>
+  </si>
+  <si>
+    <t>Not ban</t>
+  </si>
+  <si>
+    <t>Linked accounts</t>
+  </si>
 </sst>
 </file>
 
@@ -315,7 +392,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -324,6 +401,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -659,13 +749,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F8F83EB-D2AA-4A07-AAE9-D76D76655169}">
-  <dimension ref="A1:I375"/>
+  <dimension ref="A1:M375"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="9" max="9" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="25.109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="31.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -694,7 +786,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>6347039</v>
       </c>
@@ -722,8 +814,14 @@
       <c r="I2" s="2">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L2" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>7891051</v>
       </c>
@@ -751,8 +849,14 @@
       <c r="I3" s="2">
         <v>0.22500000000000001</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L3" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>7891361</v>
       </c>
@@ -780,8 +884,14 @@
       <c r="I4" s="2">
         <v>0.11042944785276074</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L4" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>7892480</v>
       </c>
@@ -809,8 +919,14 @@
       <c r="I5" s="2">
         <v>6.0606060606060608E-2</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L5" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="M5" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>7910811</v>
       </c>
@@ -838,8 +954,10 @@
       <c r="I6" s="2">
         <v>1.8828451882845189E-2</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>7928763</v>
       </c>
@@ -868,7 +986,7 @@
         <v>5.5E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7973914</v>
       </c>
@@ -897,7 +1015,7 @@
         <v>0.10526315789473684</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8000768</v>
       </c>
@@ -925,8 +1043,11 @@
       <c r="I9" s="2">
         <v>6.8669527896995708E-2</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L9" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8024534</v>
       </c>
@@ -955,7 +1076,7 @@
         <v>0.15254237288135594</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>8055025</v>
       </c>
@@ -984,7 +1105,7 @@
         <v>7.3170731707317069E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>8063461</v>
       </c>
@@ -1012,8 +1133,14 @@
       <c r="I12" s="2">
         <v>8.3333333333333329E-2</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L12" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="M12" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>8104791</v>
       </c>
@@ -1041,8 +1168,14 @@
       <c r="I13" s="2">
         <v>0.13698630136986301</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L13" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="M13" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>8121350</v>
       </c>
@@ -1070,8 +1203,14 @@
       <c r="I14" s="2">
         <v>0.11702127659574468</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L14" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="M14" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>8122967</v>
       </c>
@@ -1099,8 +1238,14 @@
       <c r="I15" s="2">
         <v>8.5714285714285715E-2</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L15" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="M15" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>8134889</v>
       </c>
@@ -1128,8 +1273,14 @@
       <c r="I16" s="2">
         <v>4.3650793650793648E-2</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L16" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="M16" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>8167915</v>
       </c>
@@ -1157,8 +1308,14 @@
       <c r="I17" s="2">
         <v>9.9173553719008267E-2</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L17" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="M17" s="9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>8175554</v>
       </c>
@@ -1186,8 +1343,14 @@
       <c r="I18" s="2">
         <v>8.9285714285714288E-2</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L18" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="M18" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>8178829</v>
       </c>
@@ -1216,7 +1379,7 @@
         <v>4.6666666666666669E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>8179309</v>
       </c>
@@ -1245,7 +1408,7 @@
         <v>6.25E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>8179889</v>
       </c>
@@ -1274,7 +1437,7 @@
         <v>0.12561174551386622</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>8198452</v>
       </c>
@@ -1303,7 +1466,7 @@
         <v>4.1666666666666664E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>8200826</v>
       </c>
@@ -1332,7 +1495,7 @@
         <v>0.4268774703557312</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>8201497</v>
       </c>
@@ -1361,7 +1524,7 @@
         <v>9.1954022988505746E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>8206493</v>
       </c>
@@ -1390,7 +1553,7 @@
         <v>0.11666666666666667</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>8215221</v>
       </c>
@@ -1419,7 +1582,7 @@
         <v>0.10169491525423729</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>8226547</v>
       </c>
@@ -1448,7 +1611,7 @@
         <v>1.8062397372742199E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>8236487</v>
       </c>
@@ -1477,7 +1640,7 @@
         <v>4.9261083743842367E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>8237768</v>
       </c>
@@ -1506,7 +1669,7 @@
         <v>3.8869257950530034E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>8240793</v>
       </c>
@@ -1535,7 +1698,7 @@
         <v>2.4590163934426229E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>8247079</v>
       </c>
@@ -1564,7 +1727,7 @@
         <v>4.9327354260089683E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>8255310</v>
       </c>
@@ -11535,6 +11698,7 @@
   </sheetData>
   <autoFilter ref="A1:I375" xr:uid="{4F8F83EB-D2AA-4A07-AAE9-D76D76655169}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -26651,6 +26815,15 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E87115C6-6BB2-4D82-9526-2FC57F5EA112}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61D8627E-AA06-4760-B4E8-1FE5600D753D}">
   <dimension ref="A1:A17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -26745,7 +26918,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC7BE25E-B4FC-4917-8A74-45B04404B799}">
   <dimension ref="A1:I24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -26842,7 +27015,7 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>42381392</v>
       </c>
       <c r="B4" s="5">
@@ -27074,7 +27247,7 @@
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="5">
+      <c r="A12" s="6">
         <v>42459298</v>
       </c>
       <c r="B12" s="5">
@@ -27456,7 +27629,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B10EE93B-10DA-4DBC-9E7F-6281E3B58B6A}">
   <dimension ref="A1:I20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -28050,17 +28223,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0757581A-7217-431E-B500-07289003B16D}">
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="19.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="9.6640625" customWidth="1"/>
+    <col min="8" max="8" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -28077,7 +28253,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>32318884</v>
       </c>
@@ -28100,7 +28276,7 @@
         <v>32318884,42372845,42381392,42406507,42426592,42426641,42458992,42459041,42459099,42459241,42459298,42463024,42463063,42705635,42731028,42913719,42971568,42997602,43022614,43081554,43110506,43138108,43166702,8200826,43230061,43290314,43319297,43346700,43374604,43402439,43430885,43539274,43566043,43593087,43614456,43674483,43862968,43891958,43920615,43949404,43978801,44010401</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>42372845</v>
       </c>
@@ -28119,7 +28295,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>42381392</v>
       </c>
@@ -28138,7 +28314,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>42406507</v>
       </c>
@@ -28157,7 +28333,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>42426592</v>
       </c>
@@ -28175,8 +28351,20 @@
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H6" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="J6" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="K6" s="12" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>42426641</v>
       </c>
@@ -28194,8 +28382,20 @@
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H7" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="I7" s="13">
+        <v>42</v>
+      </c>
+      <c r="J7" s="13">
+        <v>35</v>
+      </c>
+      <c r="K7" s="14">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>42458992</v>
       </c>
@@ -28213,8 +28413,21 @@
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H8" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="I8" s="13">
+        <v>51</v>
+      </c>
+      <c r="J8" s="13">
+        <v>22</v>
+      </c>
+      <c r="K8" s="14">
+        <f>I8-J8</f>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>42459041</v>
       </c>
@@ -28233,7 +28446,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>42459099</v>
       </c>
@@ -28252,7 +28465,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>42459241</v>
       </c>
@@ -28270,8 +28483,9 @@
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="J11" s="2"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>42459298</v>
       </c>
@@ -28289,8 +28503,9 @@
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="J12" s="11"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>42463024</v>
       </c>
@@ -28309,7 +28524,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>42463063</v>
       </c>
@@ -28328,7 +28543,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>42705635</v>
       </c>
@@ -28347,7 +28562,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>42731028</v>
       </c>

</xml_diff>

<commit_message>
add latest simulation script & results
</commit_message>
<xml_diff>
--- a/data/simulation_high_frequency_tier.xlsx
+++ b/data/simulation_high_frequency_tier.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wei.kc\Desktop\Adhoc\03 Sept 2026\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F281C01-F6B2-4D37-BCE7-6AAB99F4E84B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A5050C7-CDA4-415D-A30F-4C2271A49FDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="826" firstSheet="1" activeTab="1" xr2:uid="{2FEC0780-5ED5-45AE-9712-E8F411AADB37}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="109">
   <si>
     <t>user_id</t>
   </si>
@@ -256,9 +256,6 @@
     <t>&gt; 50% of total orders</t>
   </si>
   <si>
-    <t>Value</t>
-  </si>
-  <si>
     <t>Evaluation Window</t>
   </si>
   <si>
@@ -278,9 +275,6 @@
   </si>
   <si>
     <t>1-hour rolling window (3600 seconds)</t>
-  </si>
-  <si>
-    <t>Strategy  conditions</t>
   </si>
   <si>
     <t>Rule Threshold/Value</t>
@@ -419,17 +413,74 @@
     <t>Rolling 1hour flag &gt; 3</t>
   </si>
   <si>
-    <t>Forbid cash order</t>
+    <t>&gt; 5 high-frequency orders</t>
   </si>
   <si>
-    <t>&gt; 5 high-frequency orders</t>
+    <t>Strategy Condition</t>
+  </si>
+  <si>
+    <t>Rule Threshold / Value</t>
+  </si>
+  <si>
+    <t>Description &amp; Purpose</t>
+  </si>
+  <si>
+    <t>Order Creation Lag</t>
+  </si>
+  <si>
+    <t>Inter-order interval flag boundary for burst order placement.</t>
+  </si>
+  <si>
+    <t>Flagging Criteria</t>
+  </si>
+  <si>
+    <t>Minimum burst depth within a single window to trigger a flag event.</t>
+  </si>
+  <si>
+    <t>Continuous evaluation lookback window per user.</t>
+  </si>
+  <si>
+    <t>High Frequency Volume Share</t>
+  </si>
+  <si>
+    <t>Ensures enforcement targets accounts dominated by high-frequency activity.</t>
+  </si>
+  <si>
+    <t>Protects legitimate high-volume accounts with healthy completion rates.</t>
+  </si>
+  <si>
+    <t>Requires at least 4 distinct rolling 1-hour flag events.</t>
+  </si>
+  <si>
+    <t>Forbid Cash Order</t>
+  </si>
+  <si>
+    <t>Restricts payment method to block abusive cash-on-delivery order placement.</t>
+  </si>
+  <si>
+    <t>Completion Rate</t>
+  </si>
+  <si>
+    <t>Rolling 1-hour flag &gt;  3</t>
+  </si>
+  <si>
+    <t>July &amp; Aug 2026</t>
+  </si>
+  <si>
+    <t>Evaluation window</t>
+  </si>
+  <si>
+    <t>Enforcement trigger</t>
+  </si>
+  <si>
+    <t>Forbid cash order or order placing block</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -459,8 +510,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -479,8 +543,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9F3FD"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -516,12 +586,132 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF1F2329"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF1F2329"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF1F2329"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF1F2329"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDEE0E3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF1F2329"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF1F2329"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF1F2329"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDEE0E3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDEE0E3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDEE0E3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDEE0E3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDEE0E3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDEE0E3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDEE0E3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDEE0E3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDEE0E3"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -531,8 +721,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -545,9 +733,19 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -890,8 +1088,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
-        <v>84</v>
+      <c r="A1" s="13" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -929,7 +1127,7 @@
         <v>59</v>
       </c>
       <c r="F1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
@@ -982,7 +1180,7 @@
         <v>#N/A</v>
       </c>
       <c r="H3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -1053,17 +1251,17 @@
         <f>_xlfn.XLOOKUP(A6,'16 Accounts given'!$A$2:$A$17,'16 Accounts given'!$A$2:$A$17)</f>
         <v>#N/A</v>
       </c>
-      <c r="I6" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="J6" s="12" t="s">
+      <c r="I6" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="K6" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="K6" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="L6" s="12" t="s">
-        <v>81</v>
+      <c r="L6" s="10" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -1088,16 +1286,16 @@
         <f>_xlfn.XLOOKUP(A7,'16 Accounts given'!$A$2:$A$17,'16 Accounts given'!$A$2:$A$17)</f>
         <v>#N/A</v>
       </c>
-      <c r="I7" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="J7" s="13">
+      <c r="I7" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="J7" s="11">
         <v>42</v>
       </c>
-      <c r="K7" s="13">
+      <c r="K7" s="11">
         <v>35</v>
       </c>
-      <c r="L7" s="14">
+      <c r="L7" s="12">
         <v>7</v>
       </c>
     </row>
@@ -1123,16 +1321,16 @@
         <f>_xlfn.XLOOKUP(A8,'16 Accounts given'!$A$2:$A$17,'16 Accounts given'!$A$2:$A$17)</f>
         <v>#N/A</v>
       </c>
-      <c r="I8" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="J8" s="13">
+      <c r="I8" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="J8" s="11">
         <v>51</v>
       </c>
-      <c r="K8" s="13">
+      <c r="K8" s="11">
         <v>22</v>
       </c>
-      <c r="L8" s="14">
+      <c r="L8" s="12">
         <f>J8-K8</f>
         <v>29</v>
       </c>
@@ -1229,7 +1427,7 @@
         <f>_xlfn.XLOOKUP(A12,'16 Accounts given'!$A$2:$A$17,'16 Accounts given'!$A$2:$A$17)</f>
         <v>#N/A</v>
       </c>
-      <c r="K12" s="11"/>
+      <c r="K12" s="9"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13">
@@ -2026,11 +2224,11 @@
       <c r="I2" s="2">
         <v>0.1</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="M2" s="5" t="s">
-        <v>66</v>
+      <c r="M2" s="15" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
@@ -2062,7 +2260,7 @@
         <v>0.22500000000000001</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M3" s="5" t="s">
         <v>61</v>
@@ -2100,7 +2298,7 @@
         <v>62</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
@@ -2166,8 +2364,12 @@
       <c r="I6" s="2">
         <v>1.8828451882845189E-2</v>
       </c>
-      <c r="L6" s="10"/>
-      <c r="M6" s="10"/>
+      <c r="L6" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7">
@@ -2197,6 +2399,12 @@
       <c r="I7" s="2">
         <v>5.5E-2</v>
       </c>
+      <c r="L7" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="M7" s="14" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8">
@@ -2226,6 +2434,12 @@
       <c r="I8" s="2">
         <v>0.10526315789473684</v>
       </c>
+      <c r="L8" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9">
@@ -2255,9 +2469,6 @@
       <c r="I9" s="2">
         <v>6.8669527896995708E-2</v>
       </c>
-      <c r="L9" t="s">
-        <v>70</v>
-      </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10">
@@ -2316,6 +2527,9 @@
       <c r="I11" s="2">
         <v>7.3170731707317069E-2</v>
       </c>
+      <c r="L11" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12">
@@ -2345,11 +2559,11 @@
       <c r="I12" s="2">
         <v>8.3333333333333329E-2</v>
       </c>
-      <c r="L12" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="M12" s="5" t="s">
-        <v>75</v>
+      <c r="L12" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="M12" s="17" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
@@ -2380,11 +2594,11 @@
       <c r="I13" s="2">
         <v>0.13698630136986301</v>
       </c>
-      <c r="L13" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="M13" s="5" t="s">
-        <v>72</v>
+      <c r="L13" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="M13" s="19" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
@@ -2415,11 +2629,11 @@
       <c r="I14" s="2">
         <v>0.11702127659574468</v>
       </c>
-      <c r="L14" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="M14" s="5" t="s">
-        <v>91</v>
+      <c r="L14" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="M14" s="21" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
@@ -2450,11 +2664,11 @@
       <c r="I15" s="2">
         <v>8.5714285714285715E-2</v>
       </c>
-      <c r="L15" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="M15" s="5" t="s">
-        <v>73</v>
+      <c r="L15" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="M15" s="21" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
@@ -2485,11 +2699,11 @@
       <c r="I16" s="2">
         <v>4.3650793650793648E-2</v>
       </c>
-      <c r="L16" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="M16" s="5" t="s">
-        <v>65</v>
+      <c r="L16" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="M16" s="21" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
@@ -2520,14 +2734,11 @@
       <c r="I17" s="2">
         <v>9.9173553719008267E-2</v>
       </c>
-      <c r="L17" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="M17" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="N17" t="s">
-        <v>88</v>
+      <c r="L17" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="M17" s="23" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
@@ -2558,11 +2769,14 @@
       <c r="I18" s="2">
         <v>8.9285714285714288E-2</v>
       </c>
-      <c r="L18" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="M18" s="17" t="s">
-        <v>89</v>
+      <c r="L18" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="M18" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="N18" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
@@ -2593,11 +2807,11 @@
       <c r="I19" s="2">
         <v>4.6666666666666669E-2</v>
       </c>
-      <c r="L19" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="M19" s="9" t="s">
-        <v>90</v>
+      <c r="L19" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="M19" s="25" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
@@ -2628,6 +2842,12 @@
       <c r="I20" s="2">
         <v>6.25E-2</v>
       </c>
+      <c r="L20" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="M20" s="27" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21">
@@ -2715,6 +2935,15 @@
       <c r="I23" s="2">
         <v>0.4268774703557312</v>
       </c>
+      <c r="L23" t="s">
+        <v>89</v>
+      </c>
+      <c r="M23" t="s">
+        <v>90</v>
+      </c>
+      <c r="N23" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24">
@@ -2744,6 +2973,15 @@
       <c r="I24" s="2">
         <v>9.1954022988505746E-2</v>
       </c>
+      <c r="L24" t="s">
+        <v>92</v>
+      </c>
+      <c r="M24" t="s">
+        <v>71</v>
+      </c>
+      <c r="N24" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25">
@@ -2773,6 +3011,15 @@
       <c r="I25" s="2">
         <v>0.11666666666666667</v>
       </c>
+      <c r="L25" t="s">
+        <v>94</v>
+      </c>
+      <c r="M25" t="s">
+        <v>88</v>
+      </c>
+      <c r="N25" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26">
@@ -2802,6 +3049,15 @@
       <c r="I26" s="2">
         <v>0.10169491525423729</v>
       </c>
+      <c r="L26" t="s">
+        <v>66</v>
+      </c>
+      <c r="M26" t="s">
+        <v>72</v>
+      </c>
+      <c r="N26" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27">
@@ -2831,6 +3087,15 @@
       <c r="I27" s="2">
         <v>1.8062397372742199E-2</v>
       </c>
+      <c r="L27" t="s">
+        <v>97</v>
+      </c>
+      <c r="M27" t="s">
+        <v>65</v>
+      </c>
+      <c r="N27" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28">
@@ -2860,6 +3125,15 @@
       <c r="I28" s="2">
         <v>4.9261083743842367E-2</v>
       </c>
+      <c r="L28" t="s">
+        <v>103</v>
+      </c>
+      <c r="M28" t="s">
+        <v>85</v>
+      </c>
+      <c r="N28" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29">
@@ -2889,6 +3163,15 @@
       <c r="I29" s="2">
         <v>3.8869257950530034E-2</v>
       </c>
+      <c r="L29" t="s">
+        <v>67</v>
+      </c>
+      <c r="M29" t="s">
+        <v>104</v>
+      </c>
+      <c r="N29" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30">
@@ -2917,6 +3200,15 @@
       </c>
       <c r="I30" s="2">
         <v>2.4590163934426229E-2</v>
+      </c>
+      <c r="L30" t="s">
+        <v>68</v>
+      </c>
+      <c r="M30" t="s">
+        <v>101</v>
+      </c>
+      <c r="N30" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>